<commit_message>
Ortak kartlar (chars:[]) full review: Speed Upgrade dil bug fix
Core Mastery/Max Health Up/Medkit zaten dogruydu (Core Mastery daha once bu
session'da incelenmisti). Speed Upgrade (4): EN alani Turkce yazilmisti, TR
belirsiz/sayisizdi ("Hareket hizi artar" -> "Kalici: Hareket hizi +50").
xlsx dosyalari guncellendi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cycloneCards.xlsx
+++ b/cycloneCards.xlsx
@@ -1375,12 +1375,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>Permanent: Movement Speed +50</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>Kalıcı: Hareket hızı +50</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Hareket hızı artar</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">

</xml_diff>